<commit_message>
LMDI: Rett skrivefeil: lokaltVirkemiddel -> lokaltLegemiddel
Omdøp namingsystem-fil og oppdater URL-referanser i Medication-profil og
LegemiddelKoderValueSet til korrekt identifikator lokaltLegemiddel. 93a9e3c83d71413fcf7d4491594c6ef17422eb3f
</commit_message>
<xml_diff>
--- a/currentbuild/ValueSet-legemiddel-koder.xlsx
+++ b/currentbuild/ValueSet-legemiddel-koder.xlsx
@@ -64,7 +64,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-20T09:01:24+00:00</t>
+    <t>2026-03-27T10:18:52+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -139,7 +139,7 @@
     <t>http://dmp.no/fhir/NamingSystem/fest-varenummer</t>
   </si>
   <si>
-    <t>http://fh.no/fhir/NamingSystem/lokaltVirkemiddel</t>
+    <t>http://fh.no/fhir/NamingSystem/lokaltLegemiddel</t>
   </si>
 </sst>
 </file>

</xml_diff>